<commit_message>
Added main draw.io file with System Life Cycle Flow Chart
Added the main draw.io file that will be used for all the flowcharts and diagrams. Completed first rendition of the System Life Cycle Flowchart. Also made minor changes to the risk traceability matrix but should still be finished.
</commit_message>
<xml_diff>
--- a/Specifications/Risk_Traceability_Matrix.xlsx
+++ b/Specifications/Risk_Traceability_Matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\NoordWes Universiteit\Mechatronics Engineering\Jaar 3\Semester 2\MCTR327\Eng_DesignProject_GantryCrane_Group-18\Specifications\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E091AAEB-E4D9-475A-B69B-89A061A07F8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C587BAA-33EE-45CB-B4E4-C5BCF3D9B3B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4CE4302D-EC5D-4A58-A53C-426CE452EC11}"/>
   </bookViews>
@@ -38,9 +38,207 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="58">
+  <si>
+    <t>Table 24  Risk Traceability Matrix BEFORE Mitigation</t>
+  </si>
+  <si>
+    <t>Risk Codes</t>
+  </si>
+  <si>
+    <t>S1</t>
+  </si>
+  <si>
+    <t>S2</t>
+  </si>
+  <si>
+    <t>L1</t>
+  </si>
+  <si>
+    <t>T1</t>
+  </si>
+  <si>
+    <t>T2</t>
+  </si>
+  <si>
+    <t>K1</t>
+  </si>
+  <si>
+    <t>K2</t>
+  </si>
+  <si>
+    <t>Score legend:</t>
+  </si>
+  <si>
+    <t>1 – 4   Low risk</t>
+  </si>
+  <si>
+    <t>5 – 9   Moderate risk</t>
+  </si>
+  <si>
+    <t>10 – 14  High risk</t>
+  </si>
+  <si>
+    <t>≥ 15   Critical risk</t>
+  </si>
+  <si>
+    <t>Instructions: Fill in Likelihood (1–5) and Impact (1–5) values in the light-blue cells. Leave cells blank if that risk category does not apply to the risk code. Score = Likelihood × Impact and is coloured automatically.</t>
+  </si>
+  <si>
+    <t>Knowledge Risk
+Score</t>
+  </si>
+  <si>
+    <t>Technical Risk
+Score</t>
+  </si>
+  <si>
+    <t>Logistic Risk
+Score</t>
+  </si>
+  <si>
+    <t>Schedule Risk
+Score</t>
+  </si>
+  <si>
+    <t>Knowledge Risk
+Impact</t>
+  </si>
+  <si>
+    <t>Knowledge Risk
+Likelihood</t>
+  </si>
+  <si>
+    <t>Technical Risk
+Impact</t>
+  </si>
+  <si>
+    <t>Technical Risk
+Likelihood</t>
+  </si>
+  <si>
+    <t>Logistic Risk
+Impact</t>
+  </si>
+  <si>
+    <t>Logistic Risk
+Likelihood</t>
+  </si>
+  <si>
+    <t>Schedule Risk
+Impact</t>
+  </si>
+  <si>
+    <t>Schedule Risk
+Likelihood</t>
+  </si>
+  <si>
+    <t>Table 25  Risk Traceability Matrix AFTER Mitigation</t>
+  </si>
+  <si>
+    <t>≥ 15     Critical risk</t>
+  </si>
+  <si>
+    <t>5 – 9    Moderate risk</t>
+  </si>
+  <si>
+    <t>1 – 4    Low risk</t>
+  </si>
+  <si>
+    <t>Score colour scale:</t>
+  </si>
+  <si>
+    <t>To embed this table in your LaTeX report: install the Excel2LaTeX add-in, select the table range, and click Convert to LaTeX. Paste the output into content/B_risk_register.tex.</t>
+  </si>
+  <si>
+    <t>Excel2LaTeX export</t>
+  </si>
+  <si>
+    <t>Click the last data row, copy it (Ctrl+C), then paste below. All formulas and formatting will be replicated. Update the Risk Code in column A.</t>
+  </si>
+  <si>
+    <t>Adding rows</t>
+  </si>
+  <si>
+    <t>Fill in BEFORE Mitigation first. After defining mitigations, copy the risk codes to AFTER Mitigation and enter the revised likelihood and impact values to show the improvement.</t>
+  </si>
+  <si>
+    <t>BEFORE / AFTER sheets</t>
+  </si>
+  <si>
+    <t>Leave a cell blank if that risk category does not apply to that risk code. The score cell will remain empty automatically.</t>
+  </si>
+  <si>
+    <t>Blank cells</t>
+  </si>
+  <si>
+    <t>Calculated automatically as Likelihood × Impact. The cell colour updates via conditional formatting:
+  Green (1–4): Low    Yellow (5–9): Moderate    Orange (10–14): High    Red (≥15): Critical</t>
+  </si>
+  <si>
+    <t>Score (auto)</t>
+  </si>
+  <si>
+    <t>Rate the consequence if the risk materialises:
+  1 = Negligible   2 = Minor   3 = Moderate   4 = Major   5 = Severe</t>
+  </si>
+  <si>
+    <t>Impact (1–5)</t>
+  </si>
+  <si>
+    <t>Rate how likely the risk is to occur:
+  1 = Very Low   2 = Low   3 = Medium   4 = High   5 = Very High</t>
+  </si>
+  <si>
+    <t>Likelihood (1–5)</t>
+  </si>
+  <si>
+    <t>Enter a unique identifier for each risk (e.g. S1, S2 for Schedule risks; L1 for Logistic; T1, T2 for Technical; K1, K2 for Knowledge). Add rows by copying a data row down.</t>
+  </si>
+  <si>
+    <t>NWU Risk Traceability Matrix – How to Use</t>
+  </si>
+  <si>
+    <t>Group Risk Impact</t>
+  </si>
+  <si>
+    <t>Group Risk Likelihood</t>
+  </si>
+  <si>
+    <t>G1</t>
+  </si>
+  <si>
+    <t>G2</t>
+  </si>
+  <si>
+    <t>L2</t>
+  </si>
+  <si>
+    <t>P1</t>
+  </si>
+  <si>
+    <t>P Risk
+Likelihood</t>
+  </si>
+  <si>
+    <t>P Risk
+Impact</t>
+  </si>
+  <si>
+    <t>Logistical Risk
+Likelihood</t>
+  </si>
+  <si>
+    <t>Logistical Risk
+Impact</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -48,16 +246,147 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <i/>
+      <sz val="8"/>
+      <color rgb="FF595959"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor rgb="FF993300"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF8C00"/>
+        <bgColor rgb="FFFF6600"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFD700"/>
+        <bgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor rgb="FF008080"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDCE6F1"/>
+        <bgColor rgb="FFD9D9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9D9D9"/>
+        <bgColor rgb="FFDCE6F1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4472C4"/>
+        <bgColor rgb="FF0066CC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -65,17 +394,184 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="8">
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF000000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFD700"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF8C00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF000000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFD700"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF8C00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -405,9 +901,911 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AEDE8F47-BC4B-4B60-A383-ABA60BBBE1EE}">
-  <dimension ref="A1"/>
+  <dimension ref="B3:U60"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="3" max="3" width="4.77734375" customWidth="1"/>
+    <col min="4" max="6" width="5" customWidth="1"/>
+    <col min="7" max="7" width="5.44140625" customWidth="1"/>
+    <col min="8" max="8" width="4.88671875" customWidth="1"/>
+    <col min="9" max="10" width="4.5546875" customWidth="1"/>
+    <col min="11" max="11" width="4.6640625" customWidth="1"/>
+    <col min="12" max="12" width="5.6640625" customWidth="1"/>
+    <col min="13" max="13" width="5" customWidth="1"/>
+    <col min="14" max="14" width="4.33203125" customWidth="1"/>
+    <col min="15" max="15" width="5.109375" customWidth="1"/>
+    <col min="16" max="16" width="6.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B3" s="23" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="23"/>
+      <c r="F3" s="23"/>
+      <c r="G3" s="23"/>
+      <c r="H3" s="23"/>
+      <c r="I3" s="23"/>
+      <c r="J3" s="23"/>
+      <c r="K3" s="23"/>
+      <c r="L3" s="23"/>
+      <c r="M3" s="23"/>
+      <c r="N3" s="23"/>
+      <c r="O3" s="23"/>
+      <c r="P3" s="23"/>
+    </row>
+    <row r="4" spans="2:16" ht="79.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="F4" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="G4" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="H4" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="I4" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="J4" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="K4" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="L4" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="M4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="N4" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="O4" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="P4" s="14" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B5" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" s="9">
+        <v>5</v>
+      </c>
+      <c r="D5" s="9">
+        <v>4</v>
+      </c>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="10"/>
+      <c r="H5" s="10"/>
+      <c r="I5" s="10"/>
+      <c r="J5" s="10"/>
+      <c r="K5" s="10"/>
+      <c r="L5" s="10"/>
+      <c r="M5" s="12">
+        <f t="shared" ref="M5:M13" si="0">IF(AND(C5&lt;&gt;"",D5&lt;&gt;""),C5*D5,"")</f>
+        <v>20</v>
+      </c>
+      <c r="N5" s="8" t="str">
+        <f t="shared" ref="N5:N13" si="1">IF(AND(G5&lt;&gt;"",H5&lt;&gt;""),G5*H5,"")</f>
+        <v/>
+      </c>
+      <c r="O5" s="8" t="str">
+        <f t="shared" ref="O5:O13" si="2">IF(AND(I5&lt;&gt;"",J5&lt;&gt;""),I5*J5,"")</f>
+        <v/>
+      </c>
+      <c r="P5" s="8" t="str">
+        <f t="shared" ref="P5:P13" si="3">IF(AND(K5&lt;&gt;"",L5&lt;&gt;""),K5*L5,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B6" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" s="9">
+        <v>2</v>
+      </c>
+      <c r="D6" s="9">
+        <v>3</v>
+      </c>
+      <c r="E6" s="10"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="10"/>
+      <c r="I6" s="10"/>
+      <c r="J6" s="10"/>
+      <c r="K6" s="10"/>
+      <c r="L6" s="10"/>
+      <c r="M6" s="13">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="N6" s="8" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="O6" s="8" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="P6" s="8" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="7" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B7" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="C7" s="10"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="10"/>
+      <c r="H7" s="10"/>
+      <c r="I7" s="10"/>
+      <c r="J7" s="10"/>
+      <c r="K7" s="10"/>
+      <c r="L7" s="10"/>
+      <c r="M7" s="13"/>
+      <c r="N7" s="8"/>
+      <c r="O7" s="8"/>
+      <c r="P7" s="8"/>
+    </row>
+    <row r="8" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B8" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="10"/>
+      <c r="I8" s="10"/>
+      <c r="J8" s="10"/>
+      <c r="K8" s="10"/>
+      <c r="L8" s="10"/>
+      <c r="M8" s="13"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="8"/>
+      <c r="P8" s="8"/>
+    </row>
+    <row r="9" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B9" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="9">
+        <v>3</v>
+      </c>
+      <c r="H9" s="9">
+        <v>4</v>
+      </c>
+      <c r="I9" s="10"/>
+      <c r="J9" s="10"/>
+      <c r="K9" s="10"/>
+      <c r="L9" s="10"/>
+      <c r="M9" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="N9" s="7">
+        <f t="shared" si="1"/>
+        <v>12</v>
+      </c>
+      <c r="O9" s="8" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="P9" s="8" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="10" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B10" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="10"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="10"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="9"/>
+      <c r="H10" s="9"/>
+      <c r="I10" s="10">
+        <v>4</v>
+      </c>
+      <c r="J10" s="10">
+        <v>4</v>
+      </c>
+      <c r="K10" s="10"/>
+      <c r="L10" s="10"/>
+      <c r="M10" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="N10" s="8" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="O10" s="12">
+        <f t="shared" si="2"/>
+        <v>16</v>
+      </c>
+      <c r="P10" s="8" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="11" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B11" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="C11" s="10"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="10"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="10"/>
+      <c r="H11" s="10"/>
+      <c r="I11" s="9">
+        <v>3</v>
+      </c>
+      <c r="J11" s="9">
+        <v>5</v>
+      </c>
+      <c r="K11" s="10"/>
+      <c r="L11" s="10"/>
+      <c r="M11" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="N11" s="8" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="O11" s="12">
+        <f t="shared" si="2"/>
+        <v>15</v>
+      </c>
+      <c r="P11" s="8" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="12" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B12" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="10"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="10"/>
+      <c r="H12" s="10"/>
+      <c r="I12" s="10"/>
+      <c r="J12" s="10"/>
+      <c r="K12" s="9">
+        <v>3</v>
+      </c>
+      <c r="L12" s="9">
+        <v>4</v>
+      </c>
+      <c r="M12" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="N12" s="8" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="O12" s="8" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="P12" s="7">
+        <f t="shared" si="3"/>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B13" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="10"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="10"/>
+      <c r="H13" s="10"/>
+      <c r="I13" s="10"/>
+      <c r="J13" s="10"/>
+      <c r="K13" s="9">
+        <v>3</v>
+      </c>
+      <c r="L13" s="9">
+        <v>4</v>
+      </c>
+      <c r="M13" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="N13" s="8" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="O13" s="8" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="P13" s="7">
+        <f t="shared" si="3"/>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B16" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B17" s="5"/>
+      <c r="C17" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B18" s="4"/>
+      <c r="C18" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B19" s="3"/>
+      <c r="C19" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B20" s="2"/>
+      <c r="C20" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B22" s="24" t="s">
+        <v>14</v>
+      </c>
+      <c r="C22" s="24"/>
+      <c r="D22" s="24"/>
+      <c r="E22" s="24"/>
+      <c r="F22" s="24"/>
+      <c r="G22" s="24"/>
+      <c r="H22" s="24"/>
+      <c r="I22" s="24"/>
+      <c r="J22" s="24"/>
+      <c r="K22" s="24"/>
+      <c r="L22" s="24"/>
+      <c r="M22" s="24"/>
+      <c r="N22" s="24"/>
+      <c r="O22" s="24"/>
+      <c r="P22" s="24"/>
+    </row>
+    <row r="25" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B25" s="23" t="s">
+        <v>27</v>
+      </c>
+      <c r="C25" s="23"/>
+      <c r="D25" s="23"/>
+      <c r="E25" s="23"/>
+      <c r="F25" s="23"/>
+      <c r="G25" s="23"/>
+      <c r="H25" s="23"/>
+      <c r="I25" s="23"/>
+      <c r="J25" s="23"/>
+      <c r="K25" s="23"/>
+      <c r="L25" s="23"/>
+      <c r="M25" s="23"/>
+      <c r="N25" s="23"/>
+      <c r="O25" s="23"/>
+      <c r="P25" s="23"/>
+    </row>
+    <row r="26" spans="2:16" ht="65.400000000000006" x14ac:dyDescent="0.3">
+      <c r="B26" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="C26" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="D26" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="E26" s="14"/>
+      <c r="F26" s="14"/>
+      <c r="G26" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="H26" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="I26" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="J26" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="K26" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="L26" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="M26" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="N26" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="O26" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="P26" s="14" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="27" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B27" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="C27" s="9">
+        <v>2</v>
+      </c>
+      <c r="D27" s="9">
+        <v>4</v>
+      </c>
+      <c r="E27" s="9"/>
+      <c r="F27" s="9"/>
+      <c r="G27" s="10"/>
+      <c r="H27" s="10"/>
+      <c r="I27" s="10"/>
+      <c r="J27" s="10"/>
+      <c r="K27" s="10"/>
+      <c r="L27" s="10"/>
+      <c r="M27" s="13">
+        <f t="shared" ref="M27:M33" si="4">IF(AND(C27&lt;&gt;"",D27&lt;&gt;""),C27*D27,"")</f>
+        <v>8</v>
+      </c>
+      <c r="N27" s="8" t="str">
+        <f t="shared" ref="N27:N33" si="5">IF(AND(G27&lt;&gt;"",H27&lt;&gt;""),G27*H27,"")</f>
+        <v/>
+      </c>
+      <c r="O27" s="8" t="str">
+        <f t="shared" ref="O27:O33" si="6">IF(AND(I27&lt;&gt;"",J27&lt;&gt;""),I27*J27,"")</f>
+        <v/>
+      </c>
+      <c r="P27" s="8" t="str">
+        <f t="shared" ref="P27:P33" si="7">IF(AND(K27&lt;&gt;"",L27&lt;&gt;""),K27*L27,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B28" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="C28" s="9">
+        <v>1</v>
+      </c>
+      <c r="D28" s="9">
+        <v>2</v>
+      </c>
+      <c r="E28" s="9"/>
+      <c r="F28" s="9"/>
+      <c r="G28" s="10"/>
+      <c r="H28" s="10"/>
+      <c r="I28" s="10"/>
+      <c r="J28" s="10"/>
+      <c r="K28" s="10"/>
+      <c r="L28" s="10"/>
+      <c r="M28" s="16">
+        <f t="shared" si="4"/>
+        <v>2</v>
+      </c>
+      <c r="N28" s="8" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="O28" s="8" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="P28" s="8" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="29" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B29" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="C29" s="10"/>
+      <c r="D29" s="10"/>
+      <c r="E29" s="10"/>
+      <c r="F29" s="10"/>
+      <c r="G29" s="9">
+        <v>2</v>
+      </c>
+      <c r="H29" s="9">
+        <v>2</v>
+      </c>
+      <c r="I29" s="10"/>
+      <c r="J29" s="10"/>
+      <c r="K29" s="10"/>
+      <c r="L29" s="10"/>
+      <c r="M29" s="8" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="N29" s="16">
+        <f t="shared" si="5"/>
+        <v>4</v>
+      </c>
+      <c r="O29" s="8" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="P29" s="8" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="30" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B30" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="C30" s="10"/>
+      <c r="D30" s="10"/>
+      <c r="E30" s="10"/>
+      <c r="F30" s="10"/>
+      <c r="G30" s="10"/>
+      <c r="H30" s="10"/>
+      <c r="I30" s="9">
+        <v>3</v>
+      </c>
+      <c r="J30" s="9">
+        <v>2</v>
+      </c>
+      <c r="K30" s="10"/>
+      <c r="L30" s="10"/>
+      <c r="M30" s="8" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="N30" s="8" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="O30" s="13">
+        <f t="shared" si="6"/>
+        <v>6</v>
+      </c>
+      <c r="P30" s="8" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="31" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B31" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="C31" s="10"/>
+      <c r="D31" s="10"/>
+      <c r="E31" s="10"/>
+      <c r="F31" s="10"/>
+      <c r="G31" s="10"/>
+      <c r="H31" s="10"/>
+      <c r="I31" s="9">
+        <v>3</v>
+      </c>
+      <c r="J31" s="9">
+        <v>3</v>
+      </c>
+      <c r="K31" s="10"/>
+      <c r="L31" s="10"/>
+      <c r="M31" s="8" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="N31" s="8" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="O31" s="13">
+        <f t="shared" si="6"/>
+        <v>9</v>
+      </c>
+      <c r="P31" s="8" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+    </row>
+    <row r="32" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B32" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C32" s="10"/>
+      <c r="D32" s="10"/>
+      <c r="E32" s="10"/>
+      <c r="F32" s="10"/>
+      <c r="G32" s="10"/>
+      <c r="H32" s="10"/>
+      <c r="I32" s="10"/>
+      <c r="J32" s="10"/>
+      <c r="K32" s="9">
+        <v>2</v>
+      </c>
+      <c r="L32" s="9">
+        <v>2</v>
+      </c>
+      <c r="M32" s="8" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="N32" s="8" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="O32" s="8" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="P32" s="16">
+        <f t="shared" si="7"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33" spans="2:21" x14ac:dyDescent="0.3">
+      <c r="B33" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C33" s="10"/>
+      <c r="D33" s="10"/>
+      <c r="E33" s="10"/>
+      <c r="F33" s="10"/>
+      <c r="G33" s="10"/>
+      <c r="H33" s="10"/>
+      <c r="I33" s="10"/>
+      <c r="J33" s="10"/>
+      <c r="K33" s="9">
+        <v>2</v>
+      </c>
+      <c r="L33" s="9">
+        <v>3</v>
+      </c>
+      <c r="M33" s="8" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="N33" s="8" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="O33" s="8" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="P33" s="13">
+        <f t="shared" si="7"/>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="36" spans="2:21" x14ac:dyDescent="0.3">
+      <c r="B36" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="2:21" x14ac:dyDescent="0.3">
+      <c r="B37" s="5"/>
+      <c r="C37" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="38" spans="2:21" x14ac:dyDescent="0.3">
+      <c r="B38" s="4"/>
+      <c r="C38" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="39" spans="2:21" x14ac:dyDescent="0.3">
+      <c r="B39" s="3"/>
+      <c r="C39" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="40" spans="2:21" x14ac:dyDescent="0.3">
+      <c r="B40" s="2"/>
+      <c r="C40" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="42" spans="2:21" x14ac:dyDescent="0.3">
+      <c r="B42" s="24" t="s">
+        <v>14</v>
+      </c>
+      <c r="C42" s="24"/>
+      <c r="D42" s="24"/>
+      <c r="E42" s="24"/>
+      <c r="F42" s="24"/>
+      <c r="G42" s="24"/>
+      <c r="H42" s="24"/>
+      <c r="I42" s="24"/>
+      <c r="J42" s="24"/>
+      <c r="K42" s="24"/>
+      <c r="L42" s="24"/>
+      <c r="M42" s="24"/>
+      <c r="N42" s="24"/>
+      <c r="O42" s="24"/>
+      <c r="P42" s="24"/>
+    </row>
+    <row r="45" spans="2:21" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="T45" s="25" t="s">
+        <v>47</v>
+      </c>
+      <c r="U45" s="25"/>
+    </row>
+    <row r="47" spans="2:21" ht="290.39999999999998" x14ac:dyDescent="0.3">
+      <c r="T47" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="U47" s="22" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="48" spans="2:21" ht="158.4" x14ac:dyDescent="0.3">
+      <c r="T48" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="U48" s="22" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="49" spans="20:21" ht="184.8" x14ac:dyDescent="0.3">
+      <c r="T49" s="21" t="s">
+        <v>43</v>
+      </c>
+      <c r="U49" s="22" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="50" spans="20:21" ht="356.4" x14ac:dyDescent="0.3">
+      <c r="T50" s="21" t="s">
+        <v>41</v>
+      </c>
+      <c r="U50" s="22" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="51" spans="20:21" ht="198" x14ac:dyDescent="0.3">
+      <c r="T51" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="U51" s="22" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="52" spans="20:21" ht="290.39999999999998" x14ac:dyDescent="0.3">
+      <c r="T52" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="U52" s="22" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="53" spans="20:21" ht="237.6" x14ac:dyDescent="0.3">
+      <c r="T53" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="U53" s="22" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="54" spans="20:21" ht="277.2" x14ac:dyDescent="0.3">
+      <c r="T54" s="21" t="s">
+        <v>33</v>
+      </c>
+      <c r="U54" s="22" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="56" spans="20:21" x14ac:dyDescent="0.3">
+      <c r="T56" s="21" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="57" spans="20:21" x14ac:dyDescent="0.3">
+      <c r="T57" s="20" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="58" spans="20:21" x14ac:dyDescent="0.3">
+      <c r="T58" s="19" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="59" spans="20:21" x14ac:dyDescent="0.3">
+      <c r="T59" s="18" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="60" spans="20:21" x14ac:dyDescent="0.3">
+      <c r="T60" s="17" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="B3:P3"/>
+    <mergeCell ref="B22:P22"/>
+    <mergeCell ref="B25:P25"/>
+    <mergeCell ref="B42:P42"/>
+    <mergeCell ref="T45:U45"/>
+  </mergeCells>
+  <conditionalFormatting sqref="M5:P13">
+    <cfRule type="cellIs" dxfId="7" priority="5" operator="greaterThanOrEqual">
+      <formula>15</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="6" priority="6" operator="between">
+      <formula>10</formula>
+      <formula>14</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="5" priority="7" operator="between">
+      <formula>5</formula>
+      <formula>9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="8" operator="between">
+      <formula>1</formula>
+      <formula>4</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M27:P33">
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="greaterThanOrEqual">
+      <formula>15</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="between">
+      <formula>10</formula>
+      <formula>14</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="3" operator="between">
+      <formula>5</formula>
+      <formula>9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="4" operator="between">
+      <formula>1</formula>
+      <formula>4</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
MCTR II: ICD, Design Decisions, Diagrams
Preliminary content for MCTR II
</commit_message>
<xml_diff>
--- a/Specifications/Risk_Traceability_Matrix.xlsx
+++ b/Specifications/Risk_Traceability_Matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\NoordWes Universiteit\Mechatronics Engineering\Jaar 3\Semester 2\MCTR327\Eng_DesignProject_GantryCrane_Group-18\Specifications\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9C7C40F-A505-478C-AB18-E0303D0ECE44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5CC94B6-92C0-4187-BF3F-C5D59B8E1B98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4CE4302D-EC5D-4A58-A53C-426CE452EC11}"/>
   </bookViews>
@@ -1045,15 +1045,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>18</xdr:col>
-      <xdr:colOff>457200</xdr:colOff>
+      <xdr:colOff>419100</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>142875</xdr:rowOff>
+      <xdr:rowOff>169545</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>28</xdr:col>
-      <xdr:colOff>133350</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
+      <xdr:colOff>91440</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1083,8 +1083,69 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="7448550" y="323850"/>
-          <a:ext cx="5772150" cy="2828925"/>
+          <a:off x="7410450" y="350520"/>
+          <a:ext cx="5768340" cy="2830830"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>29</xdr:col>
+      <xdr:colOff>93345</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>106680</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>32</xdr:col>
+      <xdr:colOff>234315</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="Picture 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6D769C49-B3D0-70EA-50BF-498CA0B3DDCB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="13790295" y="649605"/>
+          <a:ext cx="1969770" cy="933450"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>